<commit_message>
docs(qms): correct recording-consent gap in EM26-35, R-15 and AIA-01
The application does show the operator a recording indicator
('Listening…', 'Recording in Boardroom Mode…', elapsed time —
frontend/components/LiveTranscription.tsx, BoardroomView.tsx). The
earlier search looked in frontend/src, which does not exist. The gap is
restated as no consent step and no notice for the other participants.
Rating, owner and due date unchanged; correction noted in AR-2026-008.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qms/evidence-2026/20_AI_Impact_Assessment/OFI-2026-06_Response_Finding_6_J-M.xlsx
+++ b/docs/qms/evidence-2026/20_AI_Impact_Assessment/OFI-2026-06_Response_Finding_6_J-M.xlsx
@@ -473,7 +473,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Carry out and record an AI Impact Assessment for EchoMind covering intended use, affected people, data protection and consent for recordings, accuracy, bias, transparency, human oversight, security and misuse, model licensing, environmental impact and governance. Add an AI impact assessment step to the design and development procedure (SOP-05) for every new feature, use case, model and release. Add AI-specific risks to the risk register and review them at management review. Implement the actions from the assessment, starting with a recording notice and consent guidance for meeting participants.</t>
+          <t>Carry out and record an AI Impact Assessment for EchoMind covering intended use, affected people, data protection and consent for recordings, accuracy, bias, transparency, human oversight, security and misuse, model licensing, environmental impact and governance. Add an AI impact assessment step to the design and development procedure (SOP-05) for every new feature, use case, model and release. Add AI-specific risks to the risk register and review them at management review. Implement the actions from the assessment, starting with a consent step and a notice for the people being recorded.</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -488,7 +488,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Assessment, SOP-05 revision and risk register: 20 Oct 2026, approved 20 Oct 2026. Assessment actions: recording notice and consent guidance 30 Nov 2026; bias measurement 31 Jan 2027. Effectiveness checked at the internal audit, 9–13 Nov 2026.</t>
+          <t>Assessment, SOP-05 revision and risk register: 20 Oct 2026, approved 20 Oct 2026. Assessment actions: consent step and participant notice 30 Nov 2026; bias measurement 31 Jan 2027. Effectiveness checked at the internal audit, 9–13 Nov 2026.</t>
         </is>
       </c>
     </row>

</xml_diff>